<commit_message>
Ficha sin saltos al cargar números y AO28 con el último cupón al vencimiento
- Los gráficos de la ficha se rehacen sin animación y, al rehacer la ficha, la página queda donde estaba.
- AO28: el último cupón (0,55) se paga el 31/10/2028 junto con el capital (estaba el 30/10 separado).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qDLwykKH6VmrvoEidDNCr
</commit_message>
<xml_diff>
--- a/data/flujos.xlsx
+++ b/data/flujos.xlsx
@@ -467,7 +467,6 @@
           <t>Flujos de fondos de los bonos de Bonerío Local</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr"/>
@@ -19200,7 +19199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F432"/>
+  <dimension ref="A1:F431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28691,37 +28690,15 @@
         <v>46080</v>
       </c>
       <c r="C431" s="5" t="n">
-        <v>47056</v>
+        <v>47057</v>
       </c>
       <c r="D431" s="7" t="n">
-        <v>0.53</v>
+        <v>0.55</v>
       </c>
       <c r="E431" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F431" s="8" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="432">
-      <c r="A432" t="inlineStr">
-        <is>
-          <t>AO28</t>
-        </is>
-      </c>
-      <c r="B432" s="5" t="n">
-        <v>46080</v>
-      </c>
-      <c r="C432" s="5" t="n">
-        <v>47057</v>
-      </c>
-      <c r="D432" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E432" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="F432" s="8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ficha sin saltos al cargar números y AO28 con el último cupón al vencimiento (#362)
- Los gráficos de la ficha se rehacen sin animación y, al rehacer la ficha, la página queda donde estaba.
- AO28: el último cupón (0,55) se paga el 31/10/2028 junto con el capital (estaba el 30/10 separado).


Claude-Session: https://claude.ai/code/session_013qDLwykKH6VmrvoEidDNCr

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flujos.xlsx
+++ b/data/flujos.xlsx
@@ -467,7 +467,6 @@
           <t>Flujos de fondos de los bonos de Bonerío Local</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr"/>
@@ -19200,7 +19199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F432"/>
+  <dimension ref="A1:F431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28691,37 +28690,15 @@
         <v>46080</v>
       </c>
       <c r="C431" s="5" t="n">
-        <v>47056</v>
+        <v>47057</v>
       </c>
       <c r="D431" s="7" t="n">
-        <v>0.53</v>
+        <v>0.55</v>
       </c>
       <c r="E431" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F431" s="8" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="432">
-      <c r="A432" t="inlineStr">
-        <is>
-          <t>AO28</t>
-        </is>
-      </c>
-      <c r="B432" s="5" t="n">
-        <v>46080</v>
-      </c>
-      <c r="C432" s="5" t="n">
-        <v>47057</v>
-      </c>
-      <c r="D432" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E432" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="F432" s="8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Licitaciones: resultado del 28/10 y alta de la Lecap S26F7
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MD2o8pzosad8VWYyPhonuq
</commit_message>
<xml_diff>
--- a/data/flujos.xlsx
+++ b/data/flujos.xlsx
@@ -25,10 +25,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -667,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K430"/>
+  <dimension ref="A1:K431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19184,6 +19185,49 @@
       <c r="K430" t="inlineStr">
         <is>
           <t>CER</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>S26F7</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>fija</t>
+        </is>
+      </c>
+      <c r="D431" s="5" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E431" s="5" t="n">
+        <v>46444</v>
+      </c>
+      <c r="F431" s="6" t="n">
+        <v>108.36762</v>
+      </c>
+      <c r="G431" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="H431" s="7" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="I431" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J431" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t>FIXED_RATE</t>
         </is>
       </c>
     </row>
@@ -29788,7 +29832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29807,6 +29851,16 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S26F7</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Licitaciones: resultado del 28/10 y alta de la Lecap S26F7 (#377)
Claude-Session: https://claude.ai/code/session_01MD2o8pzosad8VWYyPhonuq

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flujos.xlsx
+++ b/data/flujos.xlsx
@@ -25,10 +25,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -667,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K430"/>
+  <dimension ref="A1:K431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19184,6 +19185,49 @@
       <c r="K430" t="inlineStr">
         <is>
           <t>CER</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>S26F7</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>fija</t>
+        </is>
+      </c>
+      <c r="D431" s="5" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E431" s="5" t="n">
+        <v>46444</v>
+      </c>
+      <c r="F431" s="6" t="n">
+        <v>108.36762</v>
+      </c>
+      <c r="G431" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="H431" s="7" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="I431" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J431" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t>FIXED_RATE</t>
         </is>
       </c>
     </row>
@@ -29788,7 +29832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29807,6 +29851,16 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S26F7</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>